<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_educacion_tasas)
</commit_message>
<xml_diff>
--- a/output/graficos_educacion_tasas/plot_regional_e_matricula_a_2020_coquimbo.xlsx
+++ b/output/graficos_educacion_tasas/plot_regional_e_matricula_a_2020_coquimbo.xlsx
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-30 04:12</t>
+    <t xml:space="preserve">2026-10-05 06:34</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -866,13 +866,13 @@
         <v>35</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>47.5</v>
+        <v>47.6</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>49.8</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-2.3</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="13">

</xml_diff>